<commit_message>
Fix graph identity and scoring defects; add evidence filters
</commit_message>
<xml_diff>
--- a/data/processed/osteoclast_knowledge_graph_sources.xlsx
+++ b/data/processed/osteoclast_knowledge_graph_sources.xlsx
@@ -10188,7 +10188,7 @@
       </c>
       <c r="E141" t="inlineStr">
         <is>
-          <t>2-oxoglutarate (alpha-ketoglutarate)</t>
+          <t>L-glutamic acid</t>
         </is>
       </c>
       <c r="F141" t="inlineStr">
@@ -10223,7 +10223,7 @@
       </c>
       <c r="L141" t="inlineStr">
         <is>
-          <t>legacy_identity_pending_registry_mapping</t>
+          <t>registry_name_checked; biological_form_and_context_pending</t>
         </is>
       </c>
       <c r="M141" t="inlineStr">
@@ -10233,7 +10233,7 @@
       </c>
       <c r="N141" t="inlineStr">
         <is>
-          <t>core_legacy_annotations_unverified; generated_enrichment_quarantined</t>
+          <t>core_legacy_annotations_unverified; generated_enrichment_quarantined; name checked against https://www.ebi.ac.uk/chebi/CHEBI:16015 on 2026-09-29; not merged with CHEBI:30915</t>
         </is>
       </c>
     </row>
@@ -21664,12 +21664,12 @@
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>quarantined</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>Legacy claim; source registry resolution does not verify its mechanism, sign or experimental context.</t>
+          <t>CHEBI:16015 denotes L-glutamic acid, not alpha-ketoglutarate. Incident relationship quarantined after identity correction; reaction participants, protonation, direction and source support require re-curation. Legacy ACTIVATES/sign retained only as an unverified assertion.</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
@@ -21726,12 +21726,12 @@
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>quarantined</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>Legacy claim; source registry resolution does not verify its mechanism, sign or experimental context.</t>
+          <t>CHEBI:16015 denotes L-glutamic acid, not alpha-ketoglutarate. Incident relationship quarantined after identity correction; reaction participants, protonation, direction and source support require re-curation. Legacy ACTIVATES/sign retained only as an unverified assertion.</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
@@ -47935,7 +47935,7 @@
       </c>
       <c r="M37" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>quarantined</t>
         </is>
       </c>
       <c r="N37" t="inlineStr">
@@ -47945,7 +47945,7 @@
       </c>
       <c r="O37" t="inlineStr">
         <is>
-          <t>Recovered legacy narrative is a claim summary, not a source quotation. Exact source passage not yet verified.</t>
+          <t>Recovered legacy narrative is a claim summary, not a source quotation. Exact source passage not yet verified. CHEBI:16015 denotes L-glutamic acid, not alpha-ketoglutarate. Incident relationship quarantined after identity correction; reaction participants, protonation, direction and source support require re-curation. Legacy ACTIVATES/sign retained only as an unverified assertion.</t>
         </is>
       </c>
       <c r="P37" t="inlineStr">
@@ -48022,7 +48022,7 @@
       </c>
       <c r="M38" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>quarantined</t>
         </is>
       </c>
       <c r="N38" t="inlineStr">
@@ -48032,7 +48032,7 @@
       </c>
       <c r="O38" t="inlineStr">
         <is>
-          <t>Recovered legacy narrative is a claim summary, not a source quotation. Exact source passage not yet verified.</t>
+          <t>Recovered legacy narrative is a claim summary, not a source quotation. Exact source passage not yet verified. CHEBI:16015 denotes L-glutamic acid, not alpha-ketoglutarate. Incident relationship quarantined after identity correction; reaction participants, protonation, direction and source support require re-curation. Legacy ACTIVATES/sign retained only as an unverified assertion.</t>
         </is>
       </c>
       <c r="P38" t="inlineStr">

</xml_diff>